<commit_message>
fix: finalize CP0 workbook frozen panes
</commit_message>
<xml_diff>
--- a/waive/08-cp0_代码与功能覆盖率排除列表.xlsx
+++ b/waive/08-cp0_代码与功能覆盖率排除列表.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="代码waiver" sheetId="1" r:id="R3054ebcd8a784bce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能waiver" sheetId="6" r:id="Rb99512c7d7f842bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="代码waiver" sheetId="1" r:id="R1adb9f59b6f747c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="功能waiver" sheetId="6" r:id="Rd1ca6fb30cb04392"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>